<commit_message>
changed start time first session
</commit_message>
<xml_diff>
--- a/program.xlsx
+++ b/program.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marco/work/git/gwadw2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCAD7441-8FDD-284A-8EBB-3F8EA43E9688}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE564B29-416A-4243-9EB2-55D459B5C096}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="660" windowWidth="24040" windowHeight="14060" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="660" windowWidth="24040" windowHeight="14060" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Conference" sheetId="1" r:id="rId1"/>
@@ -810,9 +810,6 @@
     <t>pi5pm28</t>
   </si>
   <si>
-    <t>2025-05-19 18:00:00</t>
-  </si>
-  <si>
     <t>2026-05-20 21:00:00</t>
   </si>
   <si>
@@ -823,6 +820,9 @@
   </si>
   <si>
     <t>GWADW 2026</t>
+  </si>
+  <si>
+    <t>2025-05-15 18:00:00</t>
   </si>
 </sst>
 </file>
@@ -1185,7 +1185,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
@@ -1193,7 +1193,7 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
@@ -1534,10 +1534,10 @@
         <v>12</v>
       </c>
       <c r="C2" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>259</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>260</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
@@ -1548,10 +1548,10 @@
         <v>13</v>
       </c>
       <c r="C3" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>259</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>260</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
@@ -1562,10 +1562,10 @@
         <v>14</v>
       </c>
       <c r="C4" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>259</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>260</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
@@ -1576,10 +1576,10 @@
         <v>15</v>
       </c>
       <c r="C5" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>259</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>260</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
@@ -1590,10 +1590,10 @@
         <v>16</v>
       </c>
       <c r="C6" s="1" t="s">
+        <v>259</v>
+      </c>
+      <c r="D6" s="1" t="s">
         <v>260</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>261</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
@@ -1604,10 +1604,10 @@
         <v>17</v>
       </c>
       <c r="C7" s="1" t="s">
+        <v>259</v>
+      </c>
+      <c r="D7" s="1" t="s">
         <v>260</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>261</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
@@ -1618,10 +1618,10 @@
         <v>18</v>
       </c>
       <c r="C8" s="1" t="s">
+        <v>259</v>
+      </c>
+      <c r="D8" s="1" t="s">
         <v>260</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>261</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
@@ -1632,10 +1632,10 @@
         <v>19</v>
       </c>
       <c r="C9" s="1" t="s">
+        <v>259</v>
+      </c>
+      <c r="D9" s="1" t="s">
         <v>260</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>261</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
@@ -1646,10 +1646,10 @@
         <v>20</v>
       </c>
       <c r="C10" s="1" t="s">
+        <v>259</v>
+      </c>
+      <c r="D10" s="1" t="s">
         <v>260</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>261</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added 83 84 and 90
</commit_message>
<xml_diff>
--- a/program.xlsx
+++ b/program.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/razzano/VirgoWork/gwadw2026/gwadw2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8545FE49-A843-514C-BECE-ED4F7B3AFC6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{515D9B3F-764B-974E-B1FA-A4E674B1BFB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="660" windowWidth="24040" windowHeight="14060" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="660" windowWidth="24040" windowHeight="14060" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Conference" sheetId="1" r:id="rId1"/>
@@ -816,9 +816,6 @@
     <t>2025-05-15 18:00:00</t>
   </si>
   <si>
-    <t>2026-05-19 13:00:00</t>
-  </si>
-  <si>
     <t>2026-05-21 18:20:00</t>
   </si>
   <si>
@@ -835,6 +832,9 @@
   </si>
   <si>
     <t>University of Birmingham</t>
+  </si>
+  <si>
+    <t>2026-05-20 13:00:00</t>
   </si>
 </sst>
 </file>
@@ -1549,7 +1549,7 @@
         <v>260</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>261</v>
+        <v>267</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
@@ -1563,7 +1563,7 @@
         <v>260</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>261</v>
+        <v>267</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
@@ -1577,7 +1577,7 @@
         <v>260</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>261</v>
+        <v>267</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
@@ -1591,7 +1591,7 @@
         <v>260</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>261</v>
+        <v>267</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
@@ -1602,10 +1602,10 @@
         <v>16</v>
       </c>
       <c r="C6" s="1" t="s">
+        <v>267</v>
+      </c>
+      <c r="D6" s="1" t="s">
         <v>261</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>262</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
@@ -1616,10 +1616,10 @@
         <v>17</v>
       </c>
       <c r="C7" s="1" t="s">
+        <v>267</v>
+      </c>
+      <c r="D7" s="1" t="s">
         <v>261</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>262</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
@@ -1630,10 +1630,10 @@
         <v>18</v>
       </c>
       <c r="C8" s="1" t="s">
+        <v>267</v>
+      </c>
+      <c r="D8" s="1" t="s">
         <v>261</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>262</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
@@ -1644,10 +1644,10 @@
         <v>19</v>
       </c>
       <c r="C9" s="1" t="s">
+        <v>267</v>
+      </c>
+      <c r="D9" s="1" t="s">
         <v>261</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>262</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
@@ -1658,10 +1658,10 @@
         <v>20</v>
       </c>
       <c r="C10" s="1" t="s">
+        <v>267</v>
+      </c>
+      <c r="D10" s="1" t="s">
         <v>261</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>262</v>
       </c>
     </row>
   </sheetData>
@@ -2355,7 +2355,7 @@
         <v>100</v>
       </c>
       <c r="F7" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
@@ -2375,7 +2375,7 @@
         <v>101</v>
       </c>
       <c r="F8" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
@@ -2757,10 +2757,10 @@
         <v>153</v>
       </c>
       <c r="E5" t="s">
+        <v>264</v>
+      </c>
+      <c r="F5" t="s">
         <v>265</v>
-      </c>
-      <c r="F5" t="s">
-        <v>266</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
@@ -2777,10 +2777,10 @@
         <v>153</v>
       </c>
       <c r="E6" t="s">
+        <v>264</v>
+      </c>
+      <c r="F6" t="s">
         <v>265</v>
-      </c>
-      <c r="F6" t="s">
-        <v>266</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
@@ -2797,10 +2797,10 @@
         <v>153</v>
       </c>
       <c r="E7" t="s">
+        <v>264</v>
+      </c>
+      <c r="F7" t="s">
         <v>265</v>
-      </c>
-      <c r="F7" t="s">
-        <v>266</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
@@ -2817,10 +2817,10 @@
         <v>153</v>
       </c>
       <c r="E8" t="s">
+        <v>264</v>
+      </c>
+      <c r="F8" t="s">
         <v>265</v>
-      </c>
-      <c r="F8" t="s">
-        <v>266</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
@@ -2837,10 +2837,10 @@
         <v>153</v>
       </c>
       <c r="E9" t="s">
+        <v>264</v>
+      </c>
+      <c r="F9" t="s">
         <v>265</v>
-      </c>
-      <c r="F9" t="s">
-        <v>266</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
@@ -3053,10 +3053,10 @@
         <v>153</v>
       </c>
       <c r="E8" t="s">
+        <v>264</v>
+      </c>
+      <c r="F8" t="s">
         <v>265</v>
-      </c>
-      <c r="F8" t="s">
-        <v>266</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
@@ -3096,7 +3096,7 @@
         <v>188</v>
       </c>
       <c r="F10" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
updated 80 and moved 17 to second session
</commit_message>
<xml_diff>
--- a/program.xlsx
+++ b/program.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/razzano/VirgoWork/gwadw2026/gwadw2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E312E216-1DAA-804A-8C0E-35C36B0914EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CC63196-946B-6443-99E9-46A63B1142F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="660" windowWidth="24040" windowHeight="14060" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="660" windowWidth="24040" windowHeight="14060" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Conference" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="349" uniqueCount="254">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="353" uniqueCount="254">
   <si>
     <t>Key</t>
   </si>
@@ -1282,7 +1282,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="12.6640625" customWidth="1"/>
@@ -1389,6 +1389,26 @@
       </c>
       <c r="F5" t="s">
         <v>62</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>17</v>
+      </c>
+      <c r="B6">
+        <v>26</v>
+      </c>
+      <c r="C6" t="s">
+        <v>73</v>
+      </c>
+      <c r="D6" t="s">
+        <v>81</v>
+      </c>
+      <c r="E6" t="s">
+        <v>89</v>
+      </c>
+      <c r="F6" t="s">
+        <v>97</v>
       </c>
     </row>
   </sheetData>
@@ -1432,7 +1452,7 @@
         <v>3</v>
       </c>
       <c r="B2">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C2" t="s">
         <v>206</v>
@@ -1452,7 +1472,7 @@
         <v>11</v>
       </c>
       <c r="B3">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C3" t="s">
         <v>207</v>

</xml_diff>